<commit_message>
build_report: add images tab and singular/plural count accuracy
- Third sheet embeds all 100 traffic camera images with headline
  and outcome colour for easy doc inclusion
- Performance tab now includes count accuracy section (singular vs
  plural correctness among vehicle true positives)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018kgTcTHND39XzWgqapVK1j
</commit_message>
<xml_diff>
--- a/headline_report.xlsx
+++ b/headline_report.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Predictions vs GT" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Performance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Images" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -120,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -165,10 +166,32 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -243,6 +266,2486 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId50"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId51"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>52</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId52"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>53</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId53"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>54</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId54"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId55"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>56</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId56"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>57</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>58</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId58"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>60</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId59"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>61</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId60"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>62</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId61"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>63</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId62"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>64</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId63"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>65</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId64"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>66</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId65"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>67</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId66"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId67"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>69</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="68" name="Image 68" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId68"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>70</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="69" name="Image 69" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId69"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>71</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="70" name="Image 70" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId70"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="71" name="Image 71" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId71"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>73</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="72" name="Image 72" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId72"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>74</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="73" name="Image 73" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId73"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>75</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="74" name="Image 74" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId74"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="75" name="Image 75" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId75"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>77</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="76" name="Image 76" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId76"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>78</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="77" name="Image 77" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId77"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>79</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="78" name="Image 78" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId78"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>80</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="79" name="Image 79" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId79"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>81</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="80" name="Image 80" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId80"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>82</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="81" name="Image 81" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId81"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>83</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="82" name="Image 82" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId82"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>84</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="83" name="Image 83" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId83"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>85</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="84" name="Image 84" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId84"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>86</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="85" name="Image 85" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId85"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>87</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="86" name="Image 86" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId86"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>88</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="87" name="Image 87" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId87"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>89</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="88" name="Image 88" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId88"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>90</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="89" name="Image 89" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId89"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>91</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="90" name="Image 90" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId90"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>92</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="91" name="Image 91" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId91"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>93</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="92" name="Image 92" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId92"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>94</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="93" name="Image 93" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId93"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>95</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="94" name="Image 94" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId94"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>96</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="95" name="Image 95" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId95"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>97</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="96" name="Image 96" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId96"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>98</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="97" name="Image 97" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId97"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>99</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="98" name="Image 98" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId98"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>100</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="99" name="Image 99" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId99"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9154,10 +11657,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -9177,7 +11680,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Scores use corrected GT (29 GT annotation errors fixed by human review)</t>
+          <t>Corrected GT: 29 annotation errors fixed by human review</t>
         </is>
       </c>
     </row>
@@ -9234,17 +11737,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>1.00  ██████████</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>0.83  ████████</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>0.91  █████████</t>
+          <t>0.91</t>
         </is>
       </c>
       <c r="E6" s="12" t="n">
@@ -9266,17 +11769,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>1.00  ██████████</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>1.00  ██████████</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>1.00  ██████████</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="E7" s="12" t="n">
@@ -9298,17 +11801,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>0.70  ███████</t>
+          <t>0.70</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>0.93  █████████</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>0.80  ████████</t>
+          <t>0.80</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
@@ -9330,17 +11833,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>0.96  █████████</t>
+          <t>0.96</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>0.90  █████████</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>0.93  █████████</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="E9" s="12" t="n">
@@ -9439,17 +11942,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>1.00  ██████████</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>0.42  ████</t>
+          <t>0.42</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>0.59  █████</t>
+          <t>0.59</t>
         </is>
       </c>
       <c r="E14" s="12" t="n">
@@ -9471,17 +11974,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>1.00  ██████████</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>0.50  █████</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>0.67  ██████</t>
+          <t>0.67</t>
         </is>
       </c>
       <c r="E15" s="12" t="n">
@@ -9503,17 +12006,17 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>0.92  █████████</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>0.67  ██████</t>
+          <t>0.67</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>0.77  ███████</t>
+          <t>0.77</t>
         </is>
       </c>
       <c r="E16" s="12" t="n">
@@ -9535,17 +12038,17 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>0.50  █████</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>1.00  ██████████</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>0.67  ██████</t>
+          <t>0.67</t>
         </is>
       </c>
       <c r="E17" s="12" t="n">
@@ -9567,17 +12070,17 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>0.82  ████████</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>0.94  █████████</t>
+          <t>0.94</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>0.87  ████████</t>
+          <t>0.87</t>
         </is>
       </c>
       <c r="E18" s="12" t="n">
@@ -9657,36 +12160,1691 @@
     <row r="23">
       <c r="A23" s="18" t="inlineStr">
         <is>
-          <t>Legend</t>
+          <t>COUNT ACCURACY (singular vs plural — among vehicle TPs only)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
+          <t>Vehicle type</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Correct count</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Total TPs</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>police</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>0.71</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>ambulance</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>OVERALL</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>70</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>87</v>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
           <t>TP / TP* (GT-corrected TP)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>FP (predicted but wrong)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>FN (missed)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="115" customHeight="1">
+      <c r="A2" s="25" t="n">
+        <v>204</v>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="115" customHeight="1">
+      <c r="A3" s="25" t="n">
+        <v>205</v>
+      </c>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="115" customHeight="1">
+      <c r="A4" s="25" t="n">
+        <v>206</v>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Fire truck and police vehicle detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="115" customHeight="1">
+      <c r="A5" s="25" t="n">
+        <v>207</v>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="115" customHeight="1">
+      <c r="A6" s="25" t="n">
+        <v>208</v>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="115" customHeight="1">
+      <c r="A7" s="25" t="n">
+        <v>209</v>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="115" customHeight="1">
+      <c r="A8" s="25" t="n">
+        <v>210</v>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="115" customHeight="1">
+      <c r="A9" s="25" t="n">
+        <v>211</v>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles, Fire truck, and Ambulance detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="115" customHeight="1">
+      <c r="A10" s="25" t="n">
+        <v>212</v>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to crowd</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="115" customHeight="1">
+      <c r="A11" s="25" t="n">
+        <v>213</v>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="115" customHeight="1">
+      <c r="A12" s="25" t="n">
+        <v>214</v>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="115" customHeight="1">
+      <c r="A13" s="25" t="n">
+        <v>215</v>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="115" customHeight="1">
+      <c r="A14" s="25" t="n">
+        <v>216</v>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="115" customHeight="1">
+      <c r="A15" s="25" t="n">
+        <v>217</v>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="115" customHeight="1">
+      <c r="A16" s="25" t="n">
+        <v>218</v>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="115" customHeight="1">
+      <c r="A17" s="25" t="n">
+        <v>219</v>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="115" customHeight="1">
+      <c r="A18" s="25" t="n">
+        <v>220</v>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle and Ambulance detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="115" customHeight="1">
+      <c r="A19" s="25" t="n">
+        <v>221</v>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="115" customHeight="1">
+      <c r="A20" s="25" t="n">
+        <v>222</v>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="115" customHeight="1">
+      <c r="A21" s="25" t="n">
+        <v>223</v>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="115" customHeight="1">
+      <c r="A22" s="25" t="n">
+        <v>224</v>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="115" customHeight="1">
+      <c r="A23" s="25" t="n">
+        <v>225</v>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D23" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="115" customHeight="1">
+      <c r="A24" s="25" t="n">
+        <v>226</v>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D24" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="115" customHeight="1">
+      <c r="A25" s="25" t="n">
+        <v>227</v>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D25" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="115" customHeight="1">
+      <c r="A26" s="25" t="n">
+        <v>228</v>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D26" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="115" customHeight="1">
+      <c r="A27" s="25" t="n">
+        <v>229</v>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="115" customHeight="1">
+      <c r="A28" s="25" t="n">
+        <v>230</v>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D28" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="115" customHeight="1">
+      <c r="A29" s="25" t="n">
+        <v>231</v>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D29" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="115" customHeight="1">
+      <c r="A30" s="25" t="n">
+        <v>232</v>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to crowd</t>
+        </is>
+      </c>
+      <c r="D30" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="115" customHeight="1">
+      <c r="A31" s="25" t="n">
+        <v>233</v>
+      </c>
+      <c r="C31" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D31" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="115" customHeight="1">
+      <c r="A32" s="25" t="n">
+        <v>234</v>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="115" customHeight="1">
+      <c r="A33" s="25" t="n">
+        <v>235</v>
+      </c>
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D33" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="115" customHeight="1">
+      <c r="A34" s="25" t="n">
+        <v>236</v>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle and Fire truck detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="115" customHeight="1">
+      <c r="A35" s="25" t="n">
+        <v>237</v>
+      </c>
+      <c r="C35" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D35" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="115" customHeight="1">
+      <c r="A36" s="25" t="n">
+        <v>238</v>
+      </c>
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D36" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="115" customHeight="1">
+      <c r="A37" s="25" t="n">
+        <v>239</v>
+      </c>
+      <c r="C37" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D37" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="115" customHeight="1">
+      <c r="A38" s="25" t="n">
+        <v>240</v>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D38" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="115" customHeight="1">
+      <c r="A39" s="25" t="n">
+        <v>241</v>
+      </c>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to blocked road</t>
+        </is>
+      </c>
+      <c r="D39" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="115" customHeight="1">
+      <c r="A40" s="25" t="n">
+        <v>242</v>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D40" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="115" customHeight="1">
+      <c r="A41" s="25" t="n">
+        <v>243</v>
+      </c>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D41" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="115" customHeight="1">
+      <c r="A42" s="25" t="n">
+        <v>244</v>
+      </c>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="115" customHeight="1">
+      <c r="A43" s="25" t="n">
+        <v>245</v>
+      </c>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D43" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="115" customHeight="1">
+      <c r="A44" s="25" t="n">
+        <v>246</v>
+      </c>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D44" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="115" customHeight="1">
+      <c r="A45" s="25" t="n">
+        <v>247</v>
+      </c>
+      <c r="C45" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D45" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="115" customHeight="1">
+      <c r="A46" s="25" t="n">
+        <v>248</v>
+      </c>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="115" customHeight="1">
+      <c r="A47" s="25" t="n">
+        <v>249</v>
+      </c>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D47" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="115" customHeight="1">
+      <c r="A48" s="25" t="n">
+        <v>250</v>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D48" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="115" customHeight="1">
+      <c r="A49" s="25" t="n">
+        <v>251</v>
+      </c>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles and Fire truck detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D49" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="115" customHeight="1">
+      <c r="A50" s="25" t="n">
+        <v>252</v>
+      </c>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to blocked road</t>
+        </is>
+      </c>
+      <c r="D50" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="115" customHeight="1">
+      <c r="A51" s="25" t="n">
+        <v>253</v>
+      </c>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D51" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="115" customHeight="1">
+      <c r="A52" s="25" t="n">
+        <v>254</v>
+      </c>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D52" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="115" customHeight="1">
+      <c r="A53" s="25" t="n">
+        <v>255</v>
+      </c>
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>Emergency vehicles detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D53" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="115" customHeight="1">
+      <c r="A54" s="25" t="n">
+        <v>256</v>
+      </c>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="115" customHeight="1">
+      <c r="A55" s="25" t="n">
+        <v>257</v>
+      </c>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="115" customHeight="1">
+      <c r="A56" s="25" t="n">
+        <v>258</v>
+      </c>
+      <c r="C56" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D56" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="115" customHeight="1">
+      <c r="A57" s="25" t="n">
+        <v>259</v>
+      </c>
+      <c r="C57" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D57" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="115" customHeight="1">
+      <c r="A58" s="25" t="n">
+        <v>260</v>
+      </c>
+      <c r="C58" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D58" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="115" customHeight="1">
+      <c r="A59" s="25" t="n">
+        <v>261</v>
+      </c>
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D59" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="115" customHeight="1">
+      <c r="A60" s="25" t="n">
+        <v>262</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>[unavailable]</t>
+        </is>
+      </c>
+      <c r="C60" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D60" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="115" customHeight="1">
+      <c r="A61" s="25" t="n">
+        <v>263</v>
+      </c>
+      <c r="C61" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D61" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="115" customHeight="1">
+      <c r="A62" s="25" t="n">
+        <v>264</v>
+      </c>
+      <c r="C62" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D62" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="115" customHeight="1">
+      <c r="A63" s="25" t="n">
+        <v>265</v>
+      </c>
+      <c r="C63" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D63" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="115" customHeight="1">
+      <c r="A64" s="25" t="n">
+        <v>266</v>
+      </c>
+      <c r="C64" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to blocked road</t>
+        </is>
+      </c>
+      <c r="D64" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="115" customHeight="1">
+      <c r="A65" s="25" t="n">
+        <v>267</v>
+      </c>
+      <c r="C65" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D65" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="115" customHeight="1">
+      <c r="A66" s="25" t="n">
+        <v>268</v>
+      </c>
+      <c r="C66" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D66" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="115" customHeight="1">
+      <c r="A67" s="25" t="n">
+        <v>269</v>
+      </c>
+      <c r="C67" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D67" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="115" customHeight="1">
+      <c r="A68" s="25" t="n">
+        <v>270</v>
+      </c>
+      <c r="C68" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D68" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="115" customHeight="1">
+      <c r="A69" s="25" t="n">
+        <v>271</v>
+      </c>
+      <c r="C69" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D69" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="115" customHeight="1">
+      <c r="A70" s="25" t="n">
+        <v>272</v>
+      </c>
+      <c r="C70" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to blocked road</t>
+        </is>
+      </c>
+      <c r="D70" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="115" customHeight="1">
+      <c r="A71" s="25" t="n">
+        <v>273</v>
+      </c>
+      <c r="C71" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D71" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="115" customHeight="1">
+      <c r="A72" s="25" t="n">
+        <v>274</v>
+      </c>
+      <c r="C72" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D72" s="27" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="115" customHeight="1">
+      <c r="A73" s="25" t="n">
+        <v>275</v>
+      </c>
+      <c r="C73" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D73" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="115" customHeight="1">
+      <c r="A74" s="25" t="n">
+        <v>276</v>
+      </c>
+      <c r="C74" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D74" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="115" customHeight="1">
+      <c r="A75" s="25" t="n">
+        <v>277</v>
+      </c>
+      <c r="C75" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D75" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="115" customHeight="1">
+      <c r="A76" s="25" t="n">
+        <v>278</v>
+      </c>
+      <c r="C76" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D76" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="115" customHeight="1">
+      <c r="A77" s="25" t="n">
+        <v>279</v>
+      </c>
+      <c r="C77" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D77" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="115" customHeight="1">
+      <c r="A78" s="25" t="n">
+        <v>280</v>
+      </c>
+      <c r="C78" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D78" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="115" customHeight="1">
+      <c r="A79" s="25" t="n">
+        <v>281</v>
+      </c>
+      <c r="C79" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D79" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="115" customHeight="1">
+      <c r="A80" s="25" t="n">
+        <v>282</v>
+      </c>
+      <c r="C80" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D80" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="115" customHeight="1">
+      <c r="A81" s="25" t="n">
+        <v>283</v>
+      </c>
+      <c r="C81" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles, Fire trucks, and Ambulance detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D81" s="27" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="115" customHeight="1">
+      <c r="A82" s="25" t="n">
+        <v>284</v>
+      </c>
+      <c r="C82" s="26" t="inlineStr">
+        <is>
+          <t>Fire truck and Ambulance detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D82" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="115" customHeight="1">
+      <c r="A83" s="25" t="n">
+        <v>285</v>
+      </c>
+      <c r="C83" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D83" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="115" customHeight="1">
+      <c r="A84" s="25" t="n">
+        <v>286</v>
+      </c>
+      <c r="C84" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D84" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="115" customHeight="1">
+      <c r="A85" s="25" t="n">
+        <v>287</v>
+      </c>
+      <c r="C85" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D85" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="115" customHeight="1">
+      <c r="A86" s="25" t="n">
+        <v>288</v>
+      </c>
+      <c r="C86" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D86" s="29" t="inlineStr">
+        <is>
+          <t>FP+FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="115" customHeight="1">
+      <c r="A87" s="25" t="n">
+        <v>289</v>
+      </c>
+      <c r="C87" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D87" s="27" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="115" customHeight="1">
+      <c r="A88" s="25" t="n">
+        <v>290</v>
+      </c>
+      <c r="C88" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D88" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="115" customHeight="1">
+      <c r="A89" s="25" t="n">
+        <v>291</v>
+      </c>
+      <c r="C89" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to construction</t>
+        </is>
+      </c>
+      <c r="D89" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="115" customHeight="1">
+      <c r="A90" s="25" t="n">
+        <v>292</v>
+      </c>
+      <c r="C90" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D90" s="27" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="115" customHeight="1">
+      <c r="A91" s="25" t="n">
+        <v>293</v>
+      </c>
+      <c r="C91" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D91" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="115" customHeight="1">
+      <c r="A92" s="25" t="n">
+        <v>294</v>
+      </c>
+      <c r="C92" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D92" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="115" customHeight="1">
+      <c r="A93" s="25" t="n">
+        <v>295</v>
+      </c>
+      <c r="C93" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D93" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="115" customHeight="1">
+      <c r="A94" s="25" t="n">
+        <v>296</v>
+      </c>
+      <c r="C94" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle, Fire truck, and Ambulance detected responding to crash</t>
+        </is>
+      </c>
+      <c r="D94" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="115" customHeight="1">
+      <c r="A95" s="25" t="n">
+        <v>297</v>
+      </c>
+      <c r="C95" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicles detected responding to incident</t>
+        </is>
+      </c>
+      <c r="D95" s="27" t="inlineStr">
+        <is>
+          <t>FN</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="115" customHeight="1">
+      <c r="A96" s="25" t="n">
+        <v>298</v>
+      </c>
+      <c r="C96" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D96" s="27" t="inlineStr">
+        <is>
+          <t>FP</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="115" customHeight="1">
+      <c r="A97" s="25" t="n">
+        <v>299</v>
+      </c>
+      <c r="C97" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to blocked road</t>
+        </is>
+      </c>
+      <c r="D97" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="115" customHeight="1">
+      <c r="A98" s="25" t="n">
+        <v>300</v>
+      </c>
+      <c r="C98" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D98" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="115" customHeight="1">
+      <c r="A99" s="25" t="n">
+        <v>301</v>
+      </c>
+      <c r="C99" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D99" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="115" customHeight="1">
+      <c r="A100" s="25" t="n">
+        <v>302</v>
+      </c>
+      <c r="C100" s="26" t="inlineStr">
+        <is>
+          <t>Police vehicle detected responding to pulled-over vehicle</t>
+        </is>
+      </c>
+      <c r="D100" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="115" customHeight="1">
+      <c r="A101" s="25" t="n">
+        <v>303</v>
+      </c>
+      <c r="C101" s="26" t="inlineStr">
+        <is>
+          <t>No emergency vehicles visible</t>
+        </is>
+      </c>
+      <c r="D101" s="28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>